<commit_message>
added data and reorganised other data
</commit_message>
<xml_diff>
--- a/data/screening_agreement/reviewer_agreement_rayyan.xlsx
+++ b/data/screening_agreement/reviewer_agreement_rayyan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\screening_agreement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C02A59-019C-4F25-855C-819CAA3118C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DDA04C-2DC7-483C-BA3C-3BC629EEF2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BAEAB964-30E6-45DA-AD2A-F46573CA4E4F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{BAEAB964-30E6-45DA-AD2A-F46573CA4E4F}"/>
   </bookViews>
   <sheets>
     <sheet name="abstracts" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="67">
   <si>
     <t>Reviewer name</t>
   </si>
@@ -238,6 +238,9 @@
   </si>
   <si>
     <t>Round 3</t>
+  </si>
+  <si>
+    <t>mean overall</t>
   </si>
 </sst>
 </file>
@@ -590,20 +593,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{127713FE-D749-46EE-B0DE-3497415C3136}">
   <dimension ref="A1:J24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" customWidth="1"/>
+    <col min="4" max="4" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.81640625" customWidth="1"/>
     <col min="8" max="8" width="32" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -635,7 +638,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -655,7 +658,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -675,7 +678,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -701,7 +704,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -727,7 +730,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -747,7 +750,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -767,7 +770,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -793,7 +796,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -810,7 +813,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -836,7 +839,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -856,7 +859,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -888,7 +891,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -920,7 +923,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -946,7 +949,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -966,7 +969,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -992,7 +995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -1018,7 +1021,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1044,7 +1047,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1064,7 +1067,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1084,7 +1087,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1116,7 +1119,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1142,7 +1145,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1168,7 +1171,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1202,17 +1205,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD753D87-F8AB-4555-8F8D-B54A1CCDF3DC}">
-  <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.26953125" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -1246,8 +1249,11 @@
       <c r="K1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1286,8 +1292,12 @@
       <c r="K2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <f>AVERAGE(J2,J3,J7,J12,J14,J15,J16,J17,J18,J19,J20,J22,J24)</f>
+        <v>0.71004728612544155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1327,7 +1337,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1367,7 +1377,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1407,7 +1417,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1447,7 +1457,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1487,7 +1497,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1527,7 +1537,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1567,7 +1577,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1607,7 +1617,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1647,7 +1657,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1687,7 +1697,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1727,7 +1737,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1767,7 +1777,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1807,7 +1817,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -1847,7 +1857,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1887,7 +1897,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1927,7 +1937,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -1967,7 +1977,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -2007,7 +2017,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -2047,7 +2057,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -2087,7 +2097,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -2127,7 +2137,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>24</v>
       </c>

</xml_diff>